<commit_message>
updates to travel map
</commit_message>
<xml_diff>
--- a/assets/america_canada_travel/trip_and_lived_data.xlsx
+++ b/assets/america_canada_travel/trip_and_lived_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\OneDrive\Desktop\jangjdaniel.github.io\assets\america_canada_travel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88DF03A7-9B71-4473-A309-5B82F1566256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41B085E-B1B7-4F74-8A4D-A94C5D8E965C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -313,9 +313,6 @@
     <t>Missouri</t>
   </si>
   <si>
-    <t>St. Louis, Columbia, Kansas City</t>
-  </si>
-  <si>
     <t>technically stepping foot in kansas</t>
   </si>
   <si>
@@ -401,6 +398,9 @@
   </si>
   <si>
     <t>PhD</t>
+  </si>
+  <si>
+    <t>St. Louis, Columbia, Jefferson City, Kansas City</t>
   </si>
 </sst>
 </file>
@@ -787,7 +787,7 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1037,7 +1037,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B9" t="s">
         <v>66</v>
@@ -1250,13 +1250,13 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E15" t="s">
         <v>21</v>
@@ -1784,7 +1784,7 @@
         <v>94</v>
       </c>
       <c r="E30" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F30" s="2">
         <v>46159</v>
@@ -1845,16 +1845,16 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C32" t="s">
         <v>92</v>
       </c>
       <c r="D32" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E32" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F32" s="2">
         <v>46201</v>
@@ -1880,7 +1880,7 @@
         <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C33" t="s">
         <v>43</v>
@@ -1921,7 +1921,7 @@
         <v>96</v>
       </c>
       <c r="D34" t="s">
-        <v>97</v>
+        <v>126</v>
       </c>
       <c r="E34" t="s">
         <v>21</v>
@@ -1930,19 +1930,19 @@
         <v>46210</v>
       </c>
       <c r="G34" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H34" s="2">
         <v>46213</v>
       </c>
       <c r="I34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J34" t="s">
         <v>16</v>
       </c>
       <c r="K34" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
@@ -1950,22 +1950,22 @@
         <v>10</v>
       </c>
       <c r="B35" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" t="s">
         <v>98</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>99</v>
       </c>
-      <c r="D35" t="s">
-        <v>100</v>
-      </c>
       <c r="E35" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F35" s="2">
         <v>46211</v>
       </c>
       <c r="G35" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H35" s="2">
         <v>46211</v>
@@ -1985,16 +1985,16 @@
         <v>10</v>
       </c>
       <c r="B36" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" t="s">
         <v>104</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>105</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>106</v>
-      </c>
-      <c r="E36" t="s">
-        <v>107</v>
       </c>
       <c r="F36" s="2">
         <v>46213</v>
@@ -2006,7 +2006,7 @@
         <v>46216</v>
       </c>
       <c r="I36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J36" t="s">
         <v>16</v>
@@ -2020,16 +2020,16 @@
         <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C37" t="s">
         <v>82</v>
       </c>
       <c r="D37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E37" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F37" s="2">
         <v>46199</v>
@@ -2052,16 +2052,16 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C38" t="s">
         <v>60</v>
       </c>
       <c r="D38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F38" s="2">
         <v>39508</v>
@@ -2075,16 +2075,16 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>119</v>
+      </c>
+      <c r="B39" t="s">
         <v>120</v>
-      </c>
-      <c r="B39" t="s">
-        <v>121</v>
       </c>
       <c r="C39" t="s">
         <v>85</v>
       </c>
       <c r="D39" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F39" s="2">
         <v>39630</v>
@@ -2098,10 +2098,10 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
@@ -2121,10 +2121,10 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B41" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C41" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ jangjdaniel/jangjdaniel.github.io@33bb5667489a013f41b0768185070d5e447d77d0 🚀
</commit_message>
<xml_diff>
--- a/assets/america_canada_travel/trip_and_lived_data.xlsx
+++ b/assets/america_canada_travel/trip_and_lived_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\OneDrive\Desktop\jangjdaniel.github.io\assets\america_canada_travel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88DF03A7-9B71-4473-A309-5B82F1566256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41B085E-B1B7-4F74-8A4D-A94C5D8E965C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -313,9 +313,6 @@
     <t>Missouri</t>
   </si>
   <si>
-    <t>St. Louis, Columbia, Kansas City</t>
-  </si>
-  <si>
     <t>technically stepping foot in kansas</t>
   </si>
   <si>
@@ -401,6 +398,9 @@
   </si>
   <si>
     <t>PhD</t>
+  </si>
+  <si>
+    <t>St. Louis, Columbia, Jefferson City, Kansas City</t>
   </si>
 </sst>
 </file>
@@ -787,7 +787,7 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1037,7 +1037,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B9" t="s">
         <v>66</v>
@@ -1250,13 +1250,13 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E15" t="s">
         <v>21</v>
@@ -1784,7 +1784,7 @@
         <v>94</v>
       </c>
       <c r="E30" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F30" s="2">
         <v>46159</v>
@@ -1845,16 +1845,16 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C32" t="s">
         <v>92</v>
       </c>
       <c r="D32" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E32" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F32" s="2">
         <v>46201</v>
@@ -1880,7 +1880,7 @@
         <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C33" t="s">
         <v>43</v>
@@ -1921,7 +1921,7 @@
         <v>96</v>
       </c>
       <c r="D34" t="s">
-        <v>97</v>
+        <v>126</v>
       </c>
       <c r="E34" t="s">
         <v>21</v>
@@ -1930,19 +1930,19 @@
         <v>46210</v>
       </c>
       <c r="G34" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H34" s="2">
         <v>46213</v>
       </c>
       <c r="I34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J34" t="s">
         <v>16</v>
       </c>
       <c r="K34" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
@@ -1950,22 +1950,22 @@
         <v>10</v>
       </c>
       <c r="B35" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" t="s">
         <v>98</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>99</v>
       </c>
-      <c r="D35" t="s">
-        <v>100</v>
-      </c>
       <c r="E35" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F35" s="2">
         <v>46211</v>
       </c>
       <c r="G35" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H35" s="2">
         <v>46211</v>
@@ -1985,16 +1985,16 @@
         <v>10</v>
       </c>
       <c r="B36" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" t="s">
         <v>104</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>105</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>106</v>
-      </c>
-      <c r="E36" t="s">
-        <v>107</v>
       </c>
       <c r="F36" s="2">
         <v>46213</v>
@@ -2006,7 +2006,7 @@
         <v>46216</v>
       </c>
       <c r="I36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J36" t="s">
         <v>16</v>
@@ -2020,16 +2020,16 @@
         <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C37" t="s">
         <v>82</v>
       </c>
       <c r="D37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E37" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F37" s="2">
         <v>46199</v>
@@ -2052,16 +2052,16 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C38" t="s">
         <v>60</v>
       </c>
       <c r="D38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F38" s="2">
         <v>39508</v>
@@ -2075,16 +2075,16 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>119</v>
+      </c>
+      <c r="B39" t="s">
         <v>120</v>
-      </c>
-      <c r="B39" t="s">
-        <v>121</v>
       </c>
       <c r="C39" t="s">
         <v>85</v>
       </c>
       <c r="D39" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F39" s="2">
         <v>39630</v>
@@ -2098,10 +2098,10 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
@@ -2121,10 +2121,10 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B41" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C41" t="s">
         <v>30</v>

</xml_diff>